<commit_message>
Staffkin stop list: add 20 Valley businesses hiring now
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xt1LmB4zxjrkDQQPdVu1zS
</commit_message>
<xml_diff>
--- a/poster-run/staffkin-flyer-stops.xlsx
+++ b/poster-run/staffkin-flyer-stops.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="347">
   <si>
     <t xml:space="preserve">Staffkin flyer stops — Kentville, New Minas, Coldbrook, Wolfville, Grand Pré</t>
   </si>
@@ -700,19 +700,10 @@
     <t xml:space="preserve">390 Main St, Wolfville, NS B4P 1A4</t>
   </si>
   <si>
-    <t xml:space="preserve">Stop #</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Address</t>
+    <t xml:space="preserve">Hiring now (Job Bank / Indeed, checked 21 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same columns as the route tab. Visit with counter card A, or mail postcard B. "Address not posted" ones: mail via the Job Bank posting or skip. Care homes, support agencies and chains left out.</t>
   </si>
   <si>
     <t xml:space="preserve">Role hiring</t>
@@ -721,10 +712,313 @@
     <t xml:space="preserve">Posted</t>
   </si>
   <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
+    <t xml:space="preserve">Posting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">434 Main St, Wolfville, NS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counter card (A) in person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a line cook. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line cook; restaurant assistant manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeju Restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 Elm Ave, Wolfville, NS B4P 1Z9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Korean restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a chef. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">460 Main St, Wolfville, NS B4P 1E2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brewpub / restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a cook. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Li's Wok &amp; Grill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">112 Front St, Wolfville, NS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Church Brewing Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brewery / restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a supervisor. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No date on the posting; may be older.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor, server, kitchen team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tattingstone Inn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">620 Main St, Wolfville, NS B4P 1E8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boutique inn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a hotel manager. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indian restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring an assistant cook. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistant cook; server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sushi Fang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 Kentucky Ct, New Minas, NS B4N 4N1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sushi restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holland Home Leisure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8794 Commercial St, New Minas, NS B4N 3C5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot tub and pool retail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a retail floor manager. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retail floor manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slumber Inn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5534 Prospect Rd, New Minas, NS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a housekeeper. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Housekeeper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fleetworx Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64 Minas Warehouse Rd, New Minas, NS B4N 5G3 (verify)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck refrigeration repair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a refrigeration mechanic. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refrigeration mechanic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Archie's Welding Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address not posted (postal code B4N 3N4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welding and fabrication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference postcard (B) by mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a welding supervisor. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welding supervisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jyllikleen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address not posted (postal code B4N 3E6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleaning service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a cleaner. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleaner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidery / restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a server. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Server; line cook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Computerized Business Solutions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suite 500, 946 Park St, Kentville, NS B4N 3V7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT services office</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a receptionist. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receptionist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TJ's Convenience Store Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">466 Aldershot Rd, Kentville, NS B4N 3A4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convenience store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a cashier. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taylor MacLellan Cochrane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 Bridge St, Kentville, NS B4N 2E4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Law firm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a paralegal. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paralegal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Van Meekeren Farms Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">237 Thorpe Rd, Kentville, NS B4N 3V7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fruit farm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a fruit packer. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fruit packer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">King's Janitorial Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address not posted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commercial cleaning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eric Turner (snow removal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address not posted (postal code B4N 4K4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snow removal contractor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"I saw you're hiring a snow removal operator. Staffkin does the job ad, interview questions and reference checks. First job is free."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snow removal operator</t>
   </si>
   <si>
     <t xml:space="preserve">Option</t>
@@ -751,7 +1045,7 @@
     <t xml:space="preserve">B · Reference postcard (print front and back)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mail to hiring-now businesses (+8 spares)</t>
+    <t xml:space="preserve">Hiring-now businesses with no street address (+8 spares)</t>
   </si>
   <si>
     <t xml:space="preserve">C · Board poster</t>
@@ -934,7 +1228,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -985,10 +1279,6 @@
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -4102,72 +4392,888 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="13" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="C1" s="13" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="M4" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="N4" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="E1" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="13" t="s">
+      <c r="O4" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="G1" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="13" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="F5" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="G5" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="K1" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L1" s="13" t="s">
+      <c r="H5" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="M1" s="13" t="s">
-        <v>28</v>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="8"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="O5" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50309883","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8"/>
+      <c r="B6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="N6" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="O6" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50226438","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="8"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="O7" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50541786","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8"/>
+      <c r="B8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="8"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="N8" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="O8" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50549264","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8"/>
+      <c r="B9" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="8"/>
+      <c r="L9" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="O9" s="12" t="str">
+        <f aca="false">HYPERLINK("https://ca.indeed.com/Restaurants-jobs-in-Wolfville","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8"/>
+      <c r="B10" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="8"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="N10" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="O10" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50425508","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8"/>
+      <c r="B11" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="N11" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="O11" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50425895","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8"/>
+      <c r="B12" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>265</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="8"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="N12" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="O12" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50426176","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="8"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="N13" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="O13" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50549020","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8"/>
+      <c r="B14" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="8"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="N14" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="O14" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50360380","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8"/>
+      <c r="B15" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="8"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="N15" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="O15" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50493897","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8"/>
+      <c r="B16" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="8"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="N16" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="O16" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50455049","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8"/>
+      <c r="B17" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="8"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="N17" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="O17" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50443343","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8"/>
+      <c r="B18" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="8"/>
+      <c r="L18" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="M18" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="N18" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="O18" s="12" t="str">
+        <f aca="false">HYPERLINK("https://tasteofnovascotia.com/whos-hiring-2/","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8"/>
+      <c r="B19" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>303</v>
+      </c>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="8"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="O19" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50462370","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8"/>
+      <c r="B20" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="8"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="N20" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="O20" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50503629","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8"/>
+      <c r="B21" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>314</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="8"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="O21" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50351430","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8"/>
+      <c r="B22" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>319</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="8"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="O22" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50348596","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8"/>
+      <c r="B23" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="8"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="N23" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="O23" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50505984","Posting")</f>
+        <v>Posting</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8"/>
+      <c r="B24" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>328</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="8"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="N24" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="O24" s="12" t="str">
+        <f aca="false">HYPERLINK("https://www.jobbank.gc.ca/jobsearch/jobposting/50548172","Posting")</f>
+        <v>Posting</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L200" type="list">
-      <formula1>"To visit,Mailed,Dropped off,Spoke to owner,Declined,Follow up"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4192,115 +5298,115 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>233</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>234</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>235</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>236</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>237</v>
+      <c r="A1" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="B2" s="15" t="n">
+      <c r="A2" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="B2" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C2" s="15" t="n">
-        <f aca="false">COUNTIF('Staffkin stops'!G5:G263,"*(A)*")+4*COUNTIF('Staffkin stops'!G5:G263,"*5 counter*")+2*COUNTIF('Staffkin stops'!G5:G263,"3 counter*")+COUNTA('Hiring now'!D2:D201)+10</f>
-        <v>67</v>
-      </c>
-      <c r="D2" s="15" t="n">
+      <c r="C2" s="14" t="n">
+        <f aca="false">COUNTIF('Staffkin stops'!G5:G263,"*(A)*")+4*COUNTIF('Staffkin stops'!G5:G263,"*5 counter*")+2*COUNTIF('Staffkin stops'!G5:G263,"3 counter*")+COUNTIF('Hiring now'!G5:G224,"*(A)*")+10</f>
+        <v>83</v>
+      </c>
+      <c r="D2" s="14" t="n">
         <f aca="false">ROUNDUP(C2/B2,0)</f>
-        <v>34</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>239</v>
+        <v>42</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>240</v>
-      </c>
-      <c r="B3" s="15" t="n">
+      <c r="A3" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="B3" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C3" s="15" t="n">
-        <f aca="false">COUNTA('Hiring now'!D2:D201)+8</f>
-        <v>8</v>
-      </c>
-      <c r="D3" s="15" t="n">
+      <c r="C3" s="14" t="n">
+        <f aca="false">COUNTIF('Hiring now'!G5:G224,"*(B)*")+8</f>
+        <v>12</v>
+      </c>
+      <c r="D3" s="14" t="n">
         <f aca="false">ROUNDUP(C3/B3,0)</f>
-        <v>2</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>241</v>
+        <v>3</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>242</v>
-      </c>
-      <c r="B4" s="15" t="n">
+      <c r="A4" s="14" t="s">
+        <v>340</v>
+      </c>
+      <c r="B4" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="14" t="n">
         <f aca="false">COUNTIF('Staffkin stops'!G5:G263,"*(C)*")+2</f>
         <v>9</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="14" t="n">
         <f aca="false">ROUNDUP(C4/B4,0)</f>
         <v>9</v>
       </c>
-      <c r="E4" s="15" t="s">
-        <v>243</v>
+      <c r="E4" s="14" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="B5" s="15" t="n">
+      <c r="A5" s="14" t="s">
+        <v>342</v>
+      </c>
+      <c r="B5" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="14" t="n">
         <f aca="false">COUNTIF('Staffkin stops'!G5:G263,"*(D)*")*3+20</f>
         <v>77</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="14" t="n">
         <f aca="false">ROUNDUP(C5/B5,0)</f>
         <v>8</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>245</v>
+      <c r="E5" s="14" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>246</v>
+        <v>344</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">SUM(D2:D5)</f>
-        <v>53</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>247</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>248</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>